<commit_message>
vault backup: 2026-08-17 15:40:40
</commit_message>
<xml_diff>
--- a/Boms/Rapidburner.xlsx
+++ b/Boms/Rapidburner.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Boms\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EFFDAF-CC5E-4A78-AA4F-6A12750DEF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,110 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Quantity needed</t>
+  </si>
+  <si>
+    <t>Stocked</t>
+  </si>
+  <si>
+    <t>M3x12mm BHCS/SHCS</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>to secure cowl to X carriage</t>
+  </si>
+  <si>
+    <t>to secure cowl to hotend mount</t>
+  </si>
+  <si>
+    <t>to secure X carriage to toolhead from the rear</t>
+  </si>
+  <si>
+    <t>to secure rear brace to lower cowl</t>
+  </si>
+  <si>
+    <t>M3x6mm BHCS</t>
+  </si>
+  <si>
+    <t>M3x20mm BHCS/SHCS</t>
+  </si>
+  <si>
+    <t>M3x8mm BHCS/SHCS</t>
+  </si>
+  <si>
+    <t>M3x(20mm or 18mm or 14mm) BHCS</t>
+  </si>
+  <si>
+    <t>to secure extruder to hotend mount. Screw length depends on extruder and hotend mount</t>
+  </si>
+  <si>
+    <t>M3 nut preferably square over hexagonal</t>
+  </si>
+  <si>
+    <t>to secure the 20mm screw through the X carriage to the rear of the toolhead</t>
+  </si>
+  <si>
+    <t>M3x25mm BHCS/SHCS</t>
+  </si>
+  <si>
+    <t>to secure ADXL mount through cowl to X carriage (optional, preference would be for a nozzle mounted ADXL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 brass heat inserts </t>
+  </si>
+  <si>
+    <t>M3 brass heat inserts</t>
+  </si>
+  <si>
+    <t>to secure extruder to hotend mount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4010 24v blower fans </t>
+  </si>
+  <si>
+    <t>for part cooling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3010 24v axial fan </t>
+  </si>
+  <si>
+    <t>for hotend cooling</t>
+  </si>
+  <si>
+    <t>LEDs</t>
+  </si>
+  <si>
+    <t>for logo and nozzle lights (optional, can be a mixture of NeoPixels and/or Sequins)</t>
+  </si>
+  <si>
+    <t>2.5mm nylon zip ties</t>
+  </si>
+  <si>
+    <t>cable management</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +155,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +437,212 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="99.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-08-17 15:41:58
</commit_message>
<xml_diff>
--- a/Boms/Rapidburner.xlsx
+++ b/Boms/Rapidburner.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Boms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EFFDAF-CC5E-4A78-AA4F-6A12750DEF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A5E0D74-1325-4175-B03A-A51F9E2D0D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="21705" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="General BOM" sheetId="1" r:id="rId1"/>
+    <sheet name="V6 Hotend bom" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>Item</t>
   </si>
@@ -112,6 +113,12 @@
   </si>
   <si>
     <t>cable management</t>
+  </si>
+  <si>
+    <t>Umm, heat inserts</t>
+  </si>
+  <si>
+    <t>M3x16mm BHCS/SHCS</t>
   </si>
 </sst>
 </file>
@@ -645,4 +652,59 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96A4CC53-36C0-43A4-B08F-7D987E7C9D54}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>